<commit_message>
feat: claims cross-check + 4 views (Paid/Pending/Missing/Phantom) with KPIs, donut, weekly bar (Codex task 7)
Fix seed generator: bill nearly all visits so Kendall Jan yields Paid 392 / Pending 64 / Missing 9 / Phantom 3.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/samples/claims-kendall-jan-2026.xlsx
+++ b/public/samples/claims-kendall-jan-2026.xlsx
@@ -472,7 +472,7 @@
         <v>95</v>
       </c>
       <c r="K2" t="str">
-        <v>Aetna</v>
+        <v>Cigna</v>
       </c>
       <c r="L2" t="str">
         <v>paid</v>
@@ -554,7 +554,7 @@
         <v>95</v>
       </c>
       <c r="K4" t="str">
-        <v>Aetna</v>
+        <v>Medicare</v>
       </c>
       <c r="L4" t="str">
         <v>paid</v>
@@ -595,7 +595,7 @@
         <v>95</v>
       </c>
       <c r="K5" t="str">
-        <v>Medicare</v>
+        <v>Cigna</v>
       </c>
       <c r="L5" t="str">
         <v>paid</v>
@@ -677,7 +677,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="str">
-        <v>Medicare</v>
+        <v>Aetna</v>
       </c>
       <c r="L7" t="str">
         <v>submitted</v>
@@ -773,19 +773,19 @@
         <v>clm-0010</v>
       </c>
       <c r="B10" t="str">
-        <v>Teresa Ramos</v>
+        <v>Teresa Perez</v>
       </c>
       <c r="C10" t="str">
-        <v>1989-11-19</v>
+        <v>1955-03-09</v>
       </c>
       <c r="D10" t="str">
-        <v>3055550138</v>
+        <v>3055550120</v>
       </c>
       <c r="E10" t="str">
         <v>kendall</v>
       </c>
       <c r="F10" t="str">
-        <v>2026-01-27</v>
+        <v>2026-01-26</v>
       </c>
       <c r="G10" t="str">
         <v>97530</v>
@@ -797,10 +797,10 @@
         <v>150</v>
       </c>
       <c r="J10">
-        <v>78</v>
+        <v>127</v>
       </c>
       <c r="K10" t="str">
-        <v>BCBS FL</v>
+        <v>Cigna</v>
       </c>
       <c r="L10" t="str">
         <v>paid</v>
@@ -814,34 +814,34 @@
         <v>clm-0011</v>
       </c>
       <c r="B11" t="str">
-        <v>Patricia Torres</v>
+        <v>Carmen Delgado</v>
       </c>
       <c r="C11" t="str">
-        <v>1962-04-04</v>
+        <v>1949-09-06</v>
       </c>
       <c r="D11" t="str">
-        <v>3055550124</v>
+        <v>3055550144</v>
       </c>
       <c r="E11" t="str">
         <v>kendall</v>
       </c>
       <c r="F11" t="str">
-        <v>2026-01-27</v>
+        <v>2026-01-15</v>
       </c>
       <c r="G11" t="str">
-        <v>97110</v>
+        <v>97163</v>
       </c>
       <c r="H11" t="str">
-        <v>Physical therapy treatment</v>
+        <v>Physical therapy evaluation</v>
       </c>
       <c r="I11">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="J11">
-        <v>138</v>
+        <v>216</v>
       </c>
       <c r="K11" t="str">
-        <v>Cigna</v>
+        <v>Aetna</v>
       </c>
       <c r="L11" t="str">
         <v>paid</v>
@@ -855,22 +855,22 @@
         <v>clm-0012</v>
       </c>
       <c r="B12" t="str">
-        <v>Elena Morales</v>
+        <v>Rosa Suarez</v>
       </c>
       <c r="C12" t="str">
-        <v>1990-06-13</v>
+        <v>1994-07-22</v>
       </c>
       <c r="D12" t="str">
-        <v>3055550130</v>
+        <v>3055550140</v>
       </c>
       <c r="E12" t="str">
         <v>kendall</v>
       </c>
       <c r="F12" t="str">
-        <v>2026-01-13</v>
+        <v>2026-01-12</v>
       </c>
       <c r="G12" t="str">
-        <v>97530</v>
+        <v>97140</v>
       </c>
       <c r="H12" t="str">
         <v>Physical therapy treatment</v>
@@ -879,7 +879,7 @@
         <v>150</v>
       </c>
       <c r="J12">
-        <v>112</v>
+        <v>134</v>
       </c>
       <c r="K12" t="str">
         <v>BCBS FL</v>
@@ -896,19 +896,19 @@
         <v>clm-0013</v>
       </c>
       <c r="B13" t="str">
-        <v>Patricia Ortega</v>
+        <v>Camila Castillo</v>
       </c>
       <c r="C13" t="str">
-        <v>1957-07-12</v>
+        <v>1966-05-24</v>
       </c>
       <c r="D13" t="str">
-        <v>3055550142</v>
+        <v>3055550134</v>
       </c>
       <c r="E13" t="str">
         <v>kendall</v>
       </c>
       <c r="F13" t="str">
-        <v>2026-01-21</v>
+        <v>2026-01-06</v>
       </c>
       <c r="G13" t="str">
         <v>97110</v>
@@ -920,16 +920,16 @@
         <v>150</v>
       </c>
       <c r="J13">
-        <v>97</v>
+        <v>0</v>
       </c>
       <c r="K13" t="str">
-        <v>Aetna</v>
+        <v>Medicare</v>
       </c>
       <c r="L13" t="str">
-        <v>paid</v>
+        <v>submitted</v>
       </c>
       <c r="M13" t="str">
-        <v>2026-02-10</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(ext): seed overhaul — physicians, payer categories, fee-schedule amounts, denied/underpaid claims, POS errors (ext task 2)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/samples/claims-kendall-jan-2026.xlsx
+++ b/public/samples/claims-kendall-jan-2026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M13"/>
+  <dimension ref="A1:O13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -434,9 +434,15 @@
         <v>payer</v>
       </c>
       <c r="L1" t="str">
+        <v>provider</v>
+      </c>
+      <c r="M1" t="str">
+        <v>place_of_service</v>
+      </c>
+      <c r="N1" t="str">
         <v>claim_status</v>
       </c>
-      <c r="M1" t="str">
+      <c r="O1" t="str">
         <v>paid_date</v>
       </c>
     </row>
@@ -475,9 +481,15 @@
         <v>Cigna</v>
       </c>
       <c r="L2" t="str">
+        <v>Dr. Ricardo Fuentes, MD</v>
+      </c>
+      <c r="M2" t="str">
+        <v>office</v>
+      </c>
+      <c r="N2" t="str">
         <v>paid</v>
       </c>
-      <c r="M2" t="str">
+      <c r="O2" t="str">
         <v>2026-02-20</v>
       </c>
     </row>
@@ -516,9 +528,15 @@
         <v>Aetna</v>
       </c>
       <c r="L3" t="str">
+        <v>Dr. Sofia Delgado, MD</v>
+      </c>
+      <c r="M3" t="str">
+        <v>office</v>
+      </c>
+      <c r="N3" t="str">
         <v>paid</v>
       </c>
-      <c r="M3" t="str">
+      <c r="O3" t="str">
         <v>2026-02-20</v>
       </c>
     </row>
@@ -554,12 +572,18 @@
         <v>95</v>
       </c>
       <c r="K4" t="str">
-        <v>Medicare</v>
+        <v>BCBS FL Marketplace</v>
       </c>
       <c r="L4" t="str">
+        <v>Dr. Andres Villalobos, MD</v>
+      </c>
+      <c r="M4" t="str">
+        <v>office</v>
+      </c>
+      <c r="N4" t="str">
         <v>paid</v>
       </c>
-      <c r="M4" t="str">
+      <c r="O4" t="str">
         <v>2026-02-20</v>
       </c>
     </row>
@@ -598,9 +622,15 @@
         <v>Cigna</v>
       </c>
       <c r="L5" t="str">
+        <v>Dr. Elena Marquez, MD</v>
+      </c>
+      <c r="M5" t="str">
+        <v>office</v>
+      </c>
+      <c r="N5" t="str">
         <v>paid</v>
       </c>
-      <c r="M5" t="str">
+      <c r="O5" t="str">
         <v>2026-02-20</v>
       </c>
     </row>
@@ -636,12 +666,18 @@
         <v>0</v>
       </c>
       <c r="K6" t="str">
-        <v>Cigna</v>
+        <v>Medicare</v>
       </c>
       <c r="L6" t="str">
+        <v>Dr. Miguel Contreras, DO</v>
+      </c>
+      <c r="M6" t="str">
+        <v>office</v>
+      </c>
+      <c r="N6" t="str">
         <v>submitted</v>
       </c>
-      <c r="M6" t="str">
+      <c r="O6" t="str">
         <v/>
       </c>
     </row>
@@ -677,12 +713,18 @@
         <v>0</v>
       </c>
       <c r="K7" t="str">
-        <v>Aetna</v>
+        <v>Cigna</v>
       </c>
       <c r="L7" t="str">
+        <v>Dr. Miguel Contreras, DO</v>
+      </c>
+      <c r="M7" t="str">
+        <v>office</v>
+      </c>
+      <c r="N7" t="str">
         <v>submitted</v>
       </c>
-      <c r="M7" t="str">
+      <c r="O7" t="str">
         <v/>
       </c>
     </row>
@@ -721,9 +763,15 @@
         <v>Cigna</v>
       </c>
       <c r="L8" t="str">
+        <v>Dr. Ricardo Fuentes, MD</v>
+      </c>
+      <c r="M8" t="str">
+        <v>office</v>
+      </c>
+      <c r="N8" t="str">
         <v>paid</v>
       </c>
-      <c r="M8" t="str">
+      <c r="O8" t="str">
         <v>2026-02-21</v>
       </c>
     </row>
@@ -762,9 +810,15 @@
         <v>Aetna</v>
       </c>
       <c r="L9" t="str">
+        <v>Dr. Elena Marquez, MD</v>
+      </c>
+      <c r="M9" t="str">
+        <v/>
+      </c>
+      <c r="N9" t="str">
         <v>submitted</v>
       </c>
-      <c r="M9" t="str">
+      <c r="O9" t="str">
         <v/>
       </c>
     </row>
@@ -788,25 +842,31 @@
         <v>2026-01-26</v>
       </c>
       <c r="G10" t="str">
-        <v>97530</v>
+        <v>97140</v>
       </c>
       <c r="H10" t="str">
-        <v>Physical therapy treatment</v>
+        <v>Manual therapy</v>
       </c>
       <c r="I10">
         <v>150</v>
       </c>
       <c r="J10">
-        <v>127</v>
+        <v>0</v>
       </c>
       <c r="K10" t="str">
-        <v>Cigna</v>
+        <v>AmTrust Workers Comp</v>
       </c>
       <c r="L10" t="str">
-        <v>paid</v>
+        <v>Dr. Ricardo Fuentes, MD</v>
       </c>
       <c r="M10" t="str">
-        <v>2026-02-10</v>
+        <v>office</v>
+      </c>
+      <c r="N10" t="str">
+        <v>denied</v>
+      </c>
+      <c r="O10" t="str">
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -829,24 +889,30 @@
         <v>2026-01-15</v>
       </c>
       <c r="G11" t="str">
-        <v>97163</v>
+        <v>97161</v>
       </c>
       <c r="H11" t="str">
-        <v>Physical therapy evaluation</v>
+        <v>PT evaluation - low complexity</v>
       </c>
       <c r="I11">
         <v>200</v>
       </c>
       <c r="J11">
-        <v>216</v>
+        <v>85</v>
       </c>
       <c r="K11" t="str">
-        <v>Aetna</v>
+        <v>BCBS FL Marketplace</v>
       </c>
       <c r="L11" t="str">
+        <v>Dr. Miguel Contreras, DO</v>
+      </c>
+      <c r="M11" t="str">
+        <v>office</v>
+      </c>
+      <c r="N11" t="str">
         <v>paid</v>
       </c>
-      <c r="M11" t="str">
+      <c r="O11" t="str">
         <v>2026-02-10</v>
       </c>
     </row>
@@ -870,24 +936,30 @@
         <v>2026-01-12</v>
       </c>
       <c r="G12" t="str">
-        <v>97140</v>
+        <v>97530</v>
       </c>
       <c r="H12" t="str">
-        <v>Physical therapy treatment</v>
+        <v>Therapeutic activities</v>
       </c>
       <c r="I12">
         <v>150</v>
       </c>
       <c r="J12">
-        <v>134</v>
+        <v>25</v>
       </c>
       <c r="K12" t="str">
-        <v>BCBS FL</v>
+        <v>BCBS FL Marketplace</v>
       </c>
       <c r="L12" t="str">
+        <v>Dr. Miguel Contreras, DO</v>
+      </c>
+      <c r="M12" t="str">
+        <v>office</v>
+      </c>
+      <c r="N12" t="str">
         <v>paid</v>
       </c>
-      <c r="M12" t="str">
+      <c r="O12" t="str">
         <v>2026-02-10</v>
       </c>
     </row>
@@ -914,27 +986,33 @@
         <v>97110</v>
       </c>
       <c r="H13" t="str">
-        <v>Physical therapy treatment</v>
+        <v>Therapeutic exercise</v>
       </c>
       <c r="I13">
         <v>150</v>
       </c>
       <c r="J13">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="K13" t="str">
-        <v>Medicare</v>
+        <v>Aetna</v>
       </c>
       <c r="L13" t="str">
-        <v>submitted</v>
+        <v>Dr. Elena Marquez, MD</v>
       </c>
       <c r="M13" t="str">
-        <v/>
+        <v>office</v>
+      </c>
+      <c r="N13" t="str">
+        <v>paid</v>
+      </c>
+      <c r="O13" t="str">
+        <v>2026-02-10</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(r3): seed regen — multi-procedure claims, 5 real surgeons + 6 PCP split, showcase claim #066052423 (r3 task 2)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/samples/claims-kendall-jan-2026.xlsx
+++ b/public/samples/claims-kendall-jan-2026.xlsx
@@ -478,10 +478,10 @@
         <v>95</v>
       </c>
       <c r="K2" t="str">
-        <v>Cigna</v>
+        <v>BCBS FL</v>
       </c>
       <c r="L2" t="str">
-        <v>Dr. Ricardo Fuentes, MD</v>
+        <v>Arturo Corces, MD</v>
       </c>
       <c r="M2" t="str">
         <v>office</v>
@@ -525,10 +525,10 @@
         <v>95</v>
       </c>
       <c r="K3" t="str">
-        <v>Aetna</v>
+        <v>BCBS FL Marketplace</v>
       </c>
       <c r="L3" t="str">
-        <v>Dr. Sofia Delgado, MD</v>
+        <v>Liam McCarthy, MD</v>
       </c>
       <c r="M3" t="str">
         <v>office</v>
@@ -572,10 +572,10 @@
         <v>95</v>
       </c>
       <c r="K4" t="str">
-        <v>BCBS FL Marketplace</v>
+        <v>Medicare</v>
       </c>
       <c r="L4" t="str">
-        <v>Dr. Andres Villalobos, MD</v>
+        <v>Amar D. Rajadhyaksha, MD</v>
       </c>
       <c r="M4" t="str">
         <v>office</v>
@@ -619,10 +619,10 @@
         <v>95</v>
       </c>
       <c r="K5" t="str">
-        <v>Cigna</v>
+        <v>Ambetter (ACA Marketplace)</v>
       </c>
       <c r="L5" t="str">
-        <v>Dr. Elena Marquez, MD</v>
+        <v>Amar D. Rajadhyaksha, MD</v>
       </c>
       <c r="M5" t="str">
         <v>office</v>
@@ -666,10 +666,10 @@
         <v>0</v>
       </c>
       <c r="K6" t="str">
-        <v>Medicare</v>
+        <v>Zenith Insurance (Workers Comp)</v>
       </c>
       <c r="L6" t="str">
-        <v>Dr. Miguel Contreras, DO</v>
+        <v>Liam McCarthy, MD</v>
       </c>
       <c r="M6" t="str">
         <v>office</v>
@@ -713,10 +713,10 @@
         <v>0</v>
       </c>
       <c r="K7" t="str">
-        <v>Cigna</v>
+        <v>AmTrust Workers Comp</v>
       </c>
       <c r="L7" t="str">
-        <v>Dr. Miguel Contreras, DO</v>
+        <v>David Font-Rodriguez, MD</v>
       </c>
       <c r="M7" t="str">
         <v>office</v>
@@ -763,7 +763,7 @@
         <v>Cigna</v>
       </c>
       <c r="L8" t="str">
-        <v>Dr. Ricardo Fuentes, MD</v>
+        <v>Arturo Corces, MD</v>
       </c>
       <c r="M8" t="str">
         <v>office</v>
@@ -810,7 +810,7 @@
         <v>Aetna</v>
       </c>
       <c r="L9" t="str">
-        <v>Dr. Elena Marquez, MD</v>
+        <v>Mauricio Herrera, MD</v>
       </c>
       <c r="M9" t="str">
         <v/>
@@ -848,25 +848,25 @@
         <v>Manual therapy</v>
       </c>
       <c r="I10">
-        <v>150</v>
+        <v>575.87</v>
       </c>
       <c r="J10">
-        <v>0</v>
+        <v>45.7</v>
       </c>
       <c r="K10" t="str">
-        <v>AmTrust Workers Comp</v>
+        <v>Cigna</v>
       </c>
       <c r="L10" t="str">
-        <v>Dr. Ricardo Fuentes, MD</v>
+        <v>Liam McCarthy, MD</v>
       </c>
       <c r="M10" t="str">
         <v>office</v>
       </c>
       <c r="N10" t="str">
-        <v>denied</v>
+        <v>paid</v>
       </c>
       <c r="O10" t="str">
-        <v/>
+        <v>2026-02-13</v>
       </c>
     </row>
     <row r="11">
@@ -889,22 +889,22 @@
         <v>2026-01-15</v>
       </c>
       <c r="G11" t="str">
-        <v>97161</v>
+        <v>97162</v>
       </c>
       <c r="H11" t="str">
-        <v>PT evaluation - low complexity</v>
+        <v>PT evaluation - moderate complexity</v>
       </c>
       <c r="I11">
-        <v>200</v>
+        <v>1296.64</v>
       </c>
       <c r="J11">
-        <v>85</v>
+        <v>103.82</v>
       </c>
       <c r="K11" t="str">
         <v>BCBS FL Marketplace</v>
       </c>
       <c r="L11" t="str">
-        <v>Dr. Miguel Contreras, DO</v>
+        <v>Liam McCarthy, MD</v>
       </c>
       <c r="M11" t="str">
         <v>office</v>
@@ -913,7 +913,7 @@
         <v>paid</v>
       </c>
       <c r="O11" t="str">
-        <v>2026-02-10</v>
+        <v>2026-01-23</v>
       </c>
     </row>
     <row r="12">
@@ -936,22 +936,22 @@
         <v>2026-01-12</v>
       </c>
       <c r="G12" t="str">
-        <v>97530</v>
+        <v>97110</v>
       </c>
       <c r="H12" t="str">
-        <v>Therapeutic activities</v>
+        <v>Therapeutic exercise</v>
       </c>
       <c r="I12">
-        <v>150</v>
+        <v>592.76</v>
       </c>
       <c r="J12">
-        <v>25</v>
+        <v>44.06</v>
       </c>
       <c r="K12" t="str">
-        <v>BCBS FL Marketplace</v>
+        <v>Cigna</v>
       </c>
       <c r="L12" t="str">
-        <v>Dr. Miguel Contreras, DO</v>
+        <v>David Font-Rodriguez, MD</v>
       </c>
       <c r="M12" t="str">
         <v>office</v>
@@ -960,7 +960,7 @@
         <v>paid</v>
       </c>
       <c r="O12" t="str">
-        <v>2026-02-10</v>
+        <v>2026-01-20</v>
       </c>
     </row>
     <row r="13">
@@ -983,31 +983,31 @@
         <v>2026-01-06</v>
       </c>
       <c r="G13" t="str">
-        <v>97110</v>
+        <v>97140</v>
       </c>
       <c r="H13" t="str">
-        <v>Therapeutic exercise</v>
+        <v>Manual therapy</v>
       </c>
       <c r="I13">
-        <v>150</v>
+        <v>333.33</v>
       </c>
       <c r="J13">
-        <v>32</v>
+        <v>0</v>
       </c>
       <c r="K13" t="str">
         <v>Aetna</v>
       </c>
       <c r="L13" t="str">
-        <v>Dr. Elena Marquez, MD</v>
+        <v>Amar D. Rajadhyaksha, MD</v>
       </c>
       <c r="M13" t="str">
         <v>office</v>
       </c>
       <c r="N13" t="str">
-        <v>paid</v>
+        <v>submitted</v>
       </c>
       <c r="O13" t="str">
-        <v>2026-02-10</v>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: check-in First/Middle/Last name fields; remove Specialty column from physician summary; rename 5 physicians (Marsh/Okonkwo/Whitfield/Bianchi/Sullivan, MD)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/samples/claims-kendall-jan-2026.xlsx
+++ b/public/samples/claims-kendall-jan-2026.xlsx
@@ -481,7 +481,7 @@
         <v>BCBS FL</v>
       </c>
       <c r="L2" t="str">
-        <v>Arturo Corces, MD</v>
+        <v>Steven Marsh, MD</v>
       </c>
       <c r="M2" t="str">
         <v>office</v>
@@ -528,7 +528,7 @@
         <v>BCBS FL Marketplace</v>
       </c>
       <c r="L3" t="str">
-        <v>Liam McCarthy, MD</v>
+        <v>Michael Bianchi, MD</v>
       </c>
       <c r="M3" t="str">
         <v>office</v>
@@ -575,7 +575,7 @@
         <v>Medicare</v>
       </c>
       <c r="L4" t="str">
-        <v>Amar D. Rajadhyaksha, MD</v>
+        <v>Karen Sullivan, MD</v>
       </c>
       <c r="M4" t="str">
         <v>office</v>
@@ -622,7 +622,7 @@
         <v>Ambetter (ACA Marketplace)</v>
       </c>
       <c r="L5" t="str">
-        <v>Amar D. Rajadhyaksha, MD</v>
+        <v>Karen Sullivan, MD</v>
       </c>
       <c r="M5" t="str">
         <v>office</v>
@@ -669,7 +669,7 @@
         <v>Zenith Insurance (Workers Comp)</v>
       </c>
       <c r="L6" t="str">
-        <v>Liam McCarthy, MD</v>
+        <v>Michael Bianchi, MD</v>
       </c>
       <c r="M6" t="str">
         <v>office</v>
@@ -716,7 +716,7 @@
         <v>AmTrust Workers Comp</v>
       </c>
       <c r="L7" t="str">
-        <v>David Font-Rodriguez, MD</v>
+        <v>James Whitfield, MD</v>
       </c>
       <c r="M7" t="str">
         <v>office</v>
@@ -763,7 +763,7 @@
         <v>Cigna</v>
       </c>
       <c r="L8" t="str">
-        <v>Arturo Corces, MD</v>
+        <v>Steven Marsh, MD</v>
       </c>
       <c r="M8" t="str">
         <v>office</v>
@@ -810,7 +810,7 @@
         <v>Aetna</v>
       </c>
       <c r="L9" t="str">
-        <v>Mauricio Herrera, MD</v>
+        <v>Daniel Okonkwo, MD</v>
       </c>
       <c r="M9" t="str">
         <v/>
@@ -857,7 +857,7 @@
         <v>Cigna</v>
       </c>
       <c r="L10" t="str">
-        <v>Liam McCarthy, MD</v>
+        <v>Michael Bianchi, MD</v>
       </c>
       <c r="M10" t="str">
         <v>office</v>
@@ -904,7 +904,7 @@
         <v>BCBS FL Marketplace</v>
       </c>
       <c r="L11" t="str">
-        <v>Liam McCarthy, MD</v>
+        <v>Michael Bianchi, MD</v>
       </c>
       <c r="M11" t="str">
         <v>office</v>
@@ -951,7 +951,7 @@
         <v>Cigna</v>
       </c>
       <c r="L12" t="str">
-        <v>David Font-Rodriguez, MD</v>
+        <v>James Whitfield, MD</v>
       </c>
       <c r="M12" t="str">
         <v>office</v>
@@ -998,7 +998,7 @@
         <v>Aetna</v>
       </c>
       <c r="L13" t="str">
-        <v>Amar D. Rajadhyaksha, MD</v>
+        <v>Karen Sullivan, MD</v>
       </c>
       <c r="M13" t="str">
         <v>office</v>

</xml_diff>

<commit_message>
feat(dr): seed — follow-up visits produce physician E/M claims (99213/99214, serviceType physician) (dr task 2)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/samples/claims-kendall-jan-2026.xlsx
+++ b/public/samples/claims-kendall-jan-2026.xlsx
@@ -478,7 +478,7 @@
         <v>95</v>
       </c>
       <c r="K2" t="str">
-        <v>BCBS FL</v>
+        <v>BCBS FL Marketplace</v>
       </c>
       <c r="L2" t="str">
         <v>Steven Marsh, MD</v>
@@ -525,7 +525,7 @@
         <v>95</v>
       </c>
       <c r="K3" t="str">
-        <v>BCBS FL Marketplace</v>
+        <v>Cigna</v>
       </c>
       <c r="L3" t="str">
         <v>Michael Bianchi, MD</v>
@@ -572,7 +572,7 @@
         <v>95</v>
       </c>
       <c r="K4" t="str">
-        <v>Medicare</v>
+        <v>Cigna</v>
       </c>
       <c r="L4" t="str">
         <v>Karen Sullivan, MD</v>
@@ -619,7 +619,7 @@
         <v>95</v>
       </c>
       <c r="K5" t="str">
-        <v>Ambetter (ACA Marketplace)</v>
+        <v>BCBS FL Marketplace</v>
       </c>
       <c r="L5" t="str">
         <v>Karen Sullivan, MD</v>
@@ -666,7 +666,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="str">
-        <v>Zenith Insurance (Workers Comp)</v>
+        <v>BCBS FL</v>
       </c>
       <c r="L6" t="str">
         <v>Michael Bianchi, MD</v>
@@ -713,7 +713,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="str">
-        <v>AmTrust Workers Comp</v>
+        <v>BCBS FL</v>
       </c>
       <c r="L7" t="str">
         <v>James Whitfield, MD</v>

</xml_diff>

<commit_message>
feat(claims): HPP Adjudication Scrubber taxonomy
- New Partial Paid status; rename to Paid / Partial Paid / Unpaid / Underpaid / Denied
- Scrubber rules in reconcile.ts (Denied>Phantom>Unpaid>Partial Paid>Underpaid>Paid)
- Under review maps to Unpaid/Partial Paid; show plan status as secondary
- Denial code + reason on denied claims (detail + Denied tab)
- Contested badge on claims with an open contestation (derived from store)
- New Adjudication Rules page (definitions + rules) linked from Claims
- Seed: partial payments + CARC denial codes; contestations point at real denied/underpaid claims

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/samples/claims-kendall-jan-2026.xlsx
+++ b/public/samples/claims-kendall-jan-2026.xlsx
@@ -478,7 +478,7 @@
         <v>95</v>
       </c>
       <c r="K2" t="str">
-        <v>BCBS FL Marketplace</v>
+        <v>Medicare</v>
       </c>
       <c r="L2" t="str">
         <v>Steven Marsh, MD</v>
@@ -525,7 +525,7 @@
         <v>95</v>
       </c>
       <c r="K3" t="str">
-        <v>Cigna</v>
+        <v>Medicare</v>
       </c>
       <c r="L3" t="str">
         <v>Michael Bianchi, MD</v>
@@ -619,7 +619,7 @@
         <v>95</v>
       </c>
       <c r="K5" t="str">
-        <v>BCBS FL Marketplace</v>
+        <v>BCBS FL</v>
       </c>
       <c r="L5" t="str">
         <v>Karen Sullivan, MD</v>
@@ -666,7 +666,7 @@
         <v>0</v>
       </c>
       <c r="K6" t="str">
-        <v>BCBS FL</v>
+        <v>Zenith Insurance (Workers Comp)</v>
       </c>
       <c r="L6" t="str">
         <v>Michael Bianchi, MD</v>
@@ -898,7 +898,7 @@
         <v>1296.64</v>
       </c>
       <c r="J11">
-        <v>103.82</v>
+        <v>57.64</v>
       </c>
       <c r="K11" t="str">
         <v>BCBS FL Marketplace</v>
@@ -910,10 +910,10 @@
         <v>office</v>
       </c>
       <c r="N11" t="str">
-        <v>paid</v>
+        <v>submitted</v>
       </c>
       <c r="O11" t="str">
-        <v>2026-01-23</v>
+        <v/>
       </c>
     </row>
     <row r="12">

</xml_diff>